<commit_message>
📊 RSI Report — 2026-05-22 [auto]
</commit_message>
<xml_diff>
--- a/output/RSI_Screener_2026-05-22.xlsx
+++ b/output/RSI_Screener_2026-05-22.xlsx
@@ -497,7 +497,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NSE500  |  RSI Screener  |  Run: 22-May-2026 09:30 IST  |  0 stocks matched</t>
+          <t>NSE500  |  RSI Screener  |  Run: 22-May-2026 09:45 IST  |  0 stocks matched</t>
         </is>
       </c>
     </row>
@@ -546,17 +546,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Monthly RSI &gt; 60</t>
+          <t>Monthly RSI&gt;60</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Weekly RSI &gt; 60</t>
+          <t>Weekly RSI&gt;60</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Daily RSI 40–45</t>
+          <t>Daily RSI 40-45</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MicroCap250  |  RSI Screener  |  Run: 22-May-2026 09:32 IST  |  0 stocks matched</t>
+          <t>MicroCap250  |  RSI Screener  |  Run: 22-May-2026 09:47 IST  |  0 stocks matched</t>
         </is>
       </c>
     </row>
@@ -638,17 +638,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Monthly RSI &gt; 60</t>
+          <t>Monthly RSI&gt;60</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Weekly RSI &gt; 60</t>
+          <t>Weekly RSI&gt;60</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Daily RSI 40–45</t>
+          <t>Daily RSI 40-45</t>
         </is>
       </c>
     </row>

</xml_diff>